<commit_message>
feat: Enhance Gantt chart generation with progress tracking and improved Excel handling
- Updated `make-gantt.js` to read task progress from Excel and display it in the output.
- Modified `buildGanttExcel` to handle dynamic column ordering and conditional formatting for task bars.
- Improved `readTasksFromExcel` to detect and manage progress columns, ensuring accurate task data retrieval.
- Added new utility functions in `scheduler.js` for better task scheduling, including progress normalization and late task detection.
- Introduced a new `buildGantt.js` file for encapsulating Gantt chart generation logic.
- Updated Excel file handling to support new features and ensure compatibility with existing data structures.
</commit_message>
<xml_diff>
--- a/sample_B.xlsx
+++ b/sample_B.xlsx
@@ -11,7 +11,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+  <si>
+    <t>分類</t>
+  </si>
+  <si>
+    <t>作業Lv1</t>
+  </si>
+  <si>
+    <t>作業Lv2</t>
+  </si>
   <si>
     <t>タスク名</t>
   </si>
@@ -25,15 +34,30 @@
     <t>優先順位</t>
   </si>
   <si>
+    <t>開発</t>
+  </si>
+  <si>
+    <t>計画</t>
+  </si>
+  <si>
+    <t>要件</t>
+  </si>
+  <si>
     <t>要件定義</t>
   </si>
   <si>
     <t>田中</t>
   </si>
   <si>
+    <t>設計</t>
+  </si>
+  <si>
     <t>基本設計</t>
   </si>
   <si>
+    <t>実装</t>
+  </si>
+  <si>
     <t>詳細設計</t>
   </si>
   <si>
@@ -49,10 +73,28 @@
     <t>鈴木</t>
   </si>
   <si>
+    <t>テスト</t>
+  </si>
+  <si>
+    <t>検証</t>
+  </si>
+  <si>
+    <t>単体</t>
+  </si>
+  <si>
     <t>単体テスト</t>
   </si>
   <si>
+    <t>結合</t>
+  </si>
+  <si>
     <t>結合テスト</t>
+  </si>
+  <si>
+    <t>リリース</t>
+  </si>
+  <si>
+    <t>展開</t>
   </si>
   <si>
     <t>リリース作業</t>
@@ -432,14 +474,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="4" width="10" customWidth="1"/>
+    <col min="1" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -452,116 +495,197 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2">
         <v>5</v>
       </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-      <c r="D2">
+      <c r="G2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
         <v>8</v>
       </c>
-      <c r="D3">
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3">
+        <v>8</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4">
         <v>6</v>
       </c>
-      <c r="D4">
+      <c r="G4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5">
         <v>10</v>
       </c>
-      <c r="D5">
+      <c r="G5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
         <v>11</v>
       </c>
-      <c r="C6">
-        <v>7</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <v>4</v>
-      </c>
-      <c r="D7">
+      <c r="F8">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8">
-        <v>5</v>
-      </c>
-      <c r="D8">
+      <c r="G8">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9">
         <v>2</v>
       </c>
-      <c r="D9">
+      <c r="G9">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Refactor Gantt chart generation and task scheduling
- Updated `make-gantt.js` to remove project start date input and rely on assignee start dates from the input Excel file.
- Enhanced task scheduling logic in `scheduler.js` to use assignee-specific start dates.
- Introduced new functions in `holidays.js` to build a list of year-end holidays and improved holiday data handling.
- Modified `buildGantt.js` to create separate sheets for assignees and holidays in the output Excel file.
- Updated `readTasks.js` to read assignee and holiday sheets, ensuring proper validation and error handling.
- Changed the way holidays are processed and displayed in the Gantt chart.
- Updated sample Excel file to reflect changes in structure and data handling.
</commit_message>
<xml_diff>
--- a/sample_B.xlsx
+++ b/sample_B.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="工数一覧" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="担当者" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="31">
   <si>
     <t>分類</t>
   </si>
@@ -98,6 +99,12 @@
   </si>
   <si>
     <t>リリース作業</t>
+  </si>
+  <si>
+    <t>担当者名</t>
+  </si>
+  <si>
+    <t>参画開始日</t>
   </si>
 </sst>
 </file>
@@ -133,8 +140,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,11 +484,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="7" width="12" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -687,6 +690,49 @@
       </c>
       <c r="G9">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>